<commit_message>
FrozenSet·FrozenDictionary 매핑 유닛테스트 추가
</commit_message>
<xml_diff>
--- a/UnitTest/TestData/Excel1.xlsx
+++ b/UnitTest/TestData/Excel1.xlsx
@@ -600,7 +600,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H1048576"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultColWidth="8.62890625" defaultRowHeight="16.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.52"/>
@@ -736,30 +736,6 @@
         <v>22</v>
       </c>
     </row>
-    <row r="1048553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>